<commit_message>
:sparkles: feat: estudo de correlacao de features e estudo de hiperparametros
</commit_message>
<xml_diff>
--- a/data/datasets/dataset_raw_teste2.xlsx
+++ b/data/datasets/dataset_raw_teste2.xlsx
@@ -701,7 +701,7 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -3641,7 +3641,7 @@
       </c>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3781,7 @@
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -4061,7 +4061,7 @@
       </c>
       <c r="AB26" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -4341,7 +4341,7 @@
       </c>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -4481,7 +4481,7 @@
       </c>
       <c r="AB29" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -4761,7 +4761,7 @@
       </c>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -4901,7 +4901,7 @@
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -5041,7 +5041,7 @@
       </c>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -5181,7 +5181,7 @@
       </c>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -5321,7 +5321,7 @@
       </c>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -5461,7 +5461,7 @@
       </c>
       <c r="AB36" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -5601,7 +5601,7 @@
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -5741,7 +5741,7 @@
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -5881,7 +5881,7 @@
       </c>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PNES</t>
         </is>
       </c>
     </row>
@@ -6021,7 +6021,7 @@
       </c>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -6161,7 +6161,7 @@
       </c>
       <c r="AB41" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -6301,7 +6301,7 @@
       </c>
       <c r="AB42" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
       </c>
       <c r="AB43" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -6581,7 +6581,7 @@
       </c>
       <c r="AB44" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -6721,7 +6721,7 @@
       </c>
       <c r="AB45" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -6861,7 +6861,7 @@
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -7001,7 +7001,7 @@
       </c>
       <c r="AB47" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -7141,7 +7141,7 @@
       </c>
       <c r="AB48" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -7281,7 +7281,7 @@
       </c>
       <c r="AB49" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -7421,7 +7421,7 @@
       </c>
       <c r="AB50" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -7561,7 +7561,7 @@
       </c>
       <c r="AB51" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -7701,7 +7701,7 @@
       </c>
       <c r="AB52" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -7841,7 +7841,7 @@
       </c>
       <c r="AB53" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -7981,7 +7981,7 @@
       </c>
       <c r="AB54" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -8121,7 +8121,7 @@
       </c>
       <c r="AB55" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -8261,7 +8261,7 @@
       </c>
       <c r="AB56" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -8401,7 +8401,7 @@
       </c>
       <c r="AB57" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -8541,7 +8541,7 @@
       </c>
       <c r="AB58" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -8681,7 +8681,7 @@
       </c>
       <c r="AB59" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -8821,7 +8821,7 @@
       </c>
       <c r="AB60" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -8961,7 +8961,7 @@
       </c>
       <c r="AB61" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -9101,7 +9101,7 @@
       </c>
       <c r="AB62" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -9241,7 +9241,7 @@
       </c>
       <c r="AB63" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -9381,7 +9381,7 @@
       </c>
       <c r="AB64" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -9521,7 +9521,7 @@
       </c>
       <c r="AB65" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -9661,7 +9661,7 @@
       </c>
       <c r="AB66" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -9801,7 +9801,7 @@
       </c>
       <c r="AB67" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -9941,7 +9941,7 @@
       </c>
       <c r="AB68" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -10081,7 +10081,7 @@
       </c>
       <c r="AB69" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -10221,7 +10221,7 @@
       </c>
       <c r="AB70" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -10361,7 +10361,7 @@
       </c>
       <c r="AB71" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -10501,7 +10501,7 @@
       </c>
       <c r="AB72" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -10641,7 +10641,7 @@
       </c>
       <c r="AB73" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -10781,7 +10781,7 @@
       </c>
       <c r="AB74" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -10921,7 +10921,7 @@
       </c>
       <c r="AB75" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -11061,7 +11061,7 @@
       </c>
       <c r="AB76" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -11201,7 +11201,7 @@
       </c>
       <c r="AB77" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -11341,7 +11341,7 @@
       </c>
       <c r="AB78" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -11481,7 +11481,7 @@
       </c>
       <c r="AB79" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -11621,7 +11621,7 @@
       </c>
       <c r="AB80" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -11761,7 +11761,7 @@
       </c>
       <c r="AB81" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -11901,7 +11901,7 @@
       </c>
       <c r="AB82" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -12041,7 +12041,7 @@
       </c>
       <c r="AB83" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -12181,7 +12181,7 @@
       </c>
       <c r="AB84" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -12321,7 +12321,7 @@
       </c>
       <c r="AB85" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -12461,7 +12461,7 @@
       </c>
       <c r="AB86" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -12601,7 +12601,7 @@
       </c>
       <c r="AB87" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -12741,7 +12741,7 @@
       </c>
       <c r="AB88" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -12881,7 +12881,7 @@
       </c>
       <c r="AB89" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -13021,7 +13021,7 @@
       </c>
       <c r="AB90" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -13161,7 +13161,7 @@
       </c>
       <c r="AB91" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -13301,7 +13301,7 @@
       </c>
       <c r="AB92" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -13441,7 +13441,7 @@
       </c>
       <c r="AB93" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -13581,7 +13581,7 @@
       </c>
       <c r="AB94" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -13721,7 +13721,7 @@
       </c>
       <c r="AB95" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -13861,7 +13861,7 @@
       </c>
       <c r="AB96" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -14001,7 +14001,7 @@
       </c>
       <c r="AB97" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -14141,7 +14141,7 @@
       </c>
       <c r="AB98" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -14281,7 +14281,7 @@
       </c>
       <c r="AB99" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -14421,7 +14421,7 @@
       </c>
       <c r="AB100" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -14561,7 +14561,7 @@
       </c>
       <c r="AB101" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -14701,7 +14701,7 @@
       </c>
       <c r="AB102" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -14841,7 +14841,7 @@
       </c>
       <c r="AB103" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -14981,7 +14981,7 @@
       </c>
       <c r="AB104" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -15121,7 +15121,7 @@
       </c>
       <c r="AB105" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -15261,7 +15261,7 @@
       </c>
       <c r="AB106" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -15401,7 +15401,7 @@
       </c>
       <c r="AB107" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -15541,7 +15541,7 @@
       </c>
       <c r="AB108" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -15681,7 +15681,7 @@
       </c>
       <c r="AB109" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -15821,7 +15821,7 @@
       </c>
       <c r="AB110" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -15961,7 +15961,7 @@
       </c>
       <c r="AB111" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -16101,7 +16101,7 @@
       </c>
       <c r="AB112" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -16241,7 +16241,7 @@
       </c>
       <c r="AB113" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -16381,7 +16381,7 @@
       </c>
       <c r="AB114" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -16521,7 +16521,7 @@
       </c>
       <c r="AB115" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -16661,7 +16661,7 @@
       </c>
       <c r="AB116" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -16801,7 +16801,7 @@
       </c>
       <c r="AB117" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -16941,7 +16941,7 @@
       </c>
       <c r="AB118" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -17081,7 +17081,7 @@
       </c>
       <c r="AB119" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -17221,7 +17221,7 @@
       </c>
       <c r="AB120" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -17361,7 +17361,7 @@
       </c>
       <c r="AB121" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17501,7 @@
       </c>
       <c r="AB122" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -17641,7 +17641,7 @@
       </c>
       <c r="AB123" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -17781,7 +17781,7 @@
       </c>
       <c r="AB124" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -17921,7 +17921,7 @@
       </c>
       <c r="AB125" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -18061,7 +18061,7 @@
       </c>
       <c r="AB126" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -18201,7 +18201,7 @@
       </c>
       <c r="AB127" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -18341,7 +18341,7 @@
       </c>
       <c r="AB128" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -18481,7 +18481,7 @@
       </c>
       <c r="AB129" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -18621,7 +18621,7 @@
       </c>
       <c r="AB130" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -18761,7 +18761,7 @@
       </c>
       <c r="AB131" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -18901,7 +18901,7 @@
       </c>
       <c r="AB132" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -19041,7 +19041,7 @@
       </c>
       <c r="AB133" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -19181,7 +19181,7 @@
       </c>
       <c r="AB134" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -19321,7 +19321,7 @@
       </c>
       <c r="AB135" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -19461,7 +19461,7 @@
       </c>
       <c r="AB136" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -19601,7 +19601,7 @@
       </c>
       <c r="AB137" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -19741,7 +19741,7 @@
       </c>
       <c r="AB138" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -19881,7 +19881,7 @@
       </c>
       <c r="AB139" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
@@ -20021,7 +20021,7 @@
       </c>
       <c r="AB140" t="inlineStr">
         <is>
-          <t>PNES</t>
+          <t>SE</t>
         </is>
       </c>
     </row>

</xml_diff>